<commit_message>
Update Excel template and mapping to include all relational nested fields
</commit_message>
<xml_diff>
--- a/public/Template_Import_MBG.xlsx
+++ b/public/Template_Import_MBG.xlsx
@@ -397,50 +397,167 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:BA2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Username</v>
       </c>
       <c r="B1" t="str">
+        <v>ID SPPG</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Nomor BA Verval</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Tanggal BA Verval</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Status Operasional</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Tanggal Operasional</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Kode SPPG</v>
+      </c>
+      <c r="H1" t="str">
         <v>Nama SPPG</v>
       </c>
-      <c r="C1" t="str">
-        <v>Kode SPPG</v>
-      </c>
-      <c r="D1" t="str">
-        <v>No BA Verval</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Provinsi</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Kab/Kota</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Kecamatan</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Kelurahan</v>
-      </c>
       <c r="I1" t="str">
-        <v>Alamat</v>
+        <v>Provinsi SPPG</v>
       </c>
       <c r="J1" t="str">
-        <v>Status</v>
+        <v>Kab/Kota SPPG</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Kecamatan SPPG</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Kelurahan SPPG</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Alamat SPPG</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Kode Pos SPPG</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Latitude SPPG</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Longitude SPPG</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Jenis Bangunan SPPG</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Jenis SPPG</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Kasatpel Nama</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Kasatpel Email</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Kasatpel No HP</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Mitra Jenis</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Mitra Nama</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Mitra Pimpinan</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Mitra No HP</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Mitra Email</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Mitra Dukungan</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Mitra Provinsi</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Mitra Kab/Kota</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Mitra Kecamatan</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Mitra Kelurahan</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Mitra Alamat</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Mitra Kode Pos</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>Yayasan Nama</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>Yayasan NPWP</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>Yayasan Provinsi</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>Yayasan Kab/Kota</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>Yayasan Kecamatan</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>Yayasan Kelurahan</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>Yayasan Alamat</v>
+      </c>
+      <c r="AO1" t="str">
+        <v>Yayasan Kode Pos</v>
+      </c>
+      <c r="AP1" t="str">
+        <v>Yayasan Email</v>
+      </c>
+      <c r="AQ1" t="str">
+        <v>Yayasan Telepon</v>
+      </c>
+      <c r="AR1" t="str">
+        <v>Bank Nama</v>
+      </c>
+      <c r="AS1" t="str">
+        <v>Bank Nomor Rekening</v>
+      </c>
+      <c r="AT1" t="str">
+        <v>Bank Pemilik</v>
+      </c>
+      <c r="AU1" t="str">
+        <v>Bank VA Nama Bank</v>
+      </c>
+      <c r="AV1" t="str">
+        <v>Bank VA Nomor</v>
+      </c>
+      <c r="AW1" t="str">
+        <v>Bank VA Nama</v>
+      </c>
+      <c r="AX1" t="str">
+        <v>Perwakilan Nama</v>
+      </c>
+      <c r="AY1" t="str">
+        <v>Perwakilan NIK</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Perwakilan Email</v>
+      </c>
+      <c r="BA1" t="str">
+        <v>Perwakilan No HP</v>
       </c>
     </row>
     <row r="2">
@@ -448,36 +565,165 @@
         <v>sppg-bogor</v>
       </c>
       <c r="B2" t="str">
-        <v>SPPG Bogor Sukamaju</v>
+        <v>SPPG-1790731471291</v>
       </c>
       <c r="C2" t="str">
-        <v>KODE-32.01.2001</v>
+        <v>440/BA/VERVAL/JAKARTA/XII/2025</v>
       </c>
       <c r="D2" t="str">
-        <v>100/BA/VERVAL/IX/2025</v>
+        <v>30/12/2025</v>
       </c>
       <c r="E2" t="str">
+        <v>Beroperasi</v>
+      </c>
+      <c r="F2" t="str">
+        <v>6/1/2026</v>
+      </c>
+      <c r="G2" t="str">
+        <v>32.01.06.2001.15</v>
+      </c>
+      <c r="H2" t="str">
+        <v>SPPG Bogor Jonggol Sukamaju 3</v>
+      </c>
+      <c r="I2" t="str">
         <v>JAWA BARAT</v>
       </c>
-      <c r="F2" t="str">
-        <v>KAB. BOGOR</v>
-      </c>
-      <c r="G2" t="str">
+      <c r="J2" t="str">
+        <v>BOGOR</v>
+      </c>
+      <c r="K2" t="str">
         <v>JONGGOL</v>
       </c>
-      <c r="H2" t="str">
+      <c r="L2" t="str">
         <v>SUKAMAJU</v>
       </c>
-      <c r="I2" t="str">
-        <v>Jl. Raya Jonggol No. 12</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Beroperasi</v>
+      <c r="M2" t="str">
+        <v>Ciganitri Tengah No.29, RT 004, RW 003</v>
+      </c>
+      <c r="N2" t="str">
+        <v>40287</v>
+      </c>
+      <c r="O2" t="str">
+        <v>-6.9690927</v>
+      </c>
+      <c r="P2" t="str">
+        <v>107.6489864</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Rumah Tinggal</v>
+      </c>
+      <c r="R2" t="str">
+        <v>SPPG Mitra</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Ginanjar Surya Hardiansyah</v>
+      </c>
+      <c r="T2" t="str">
+        <v>ginanjarsuryah@gmail.com</v>
+      </c>
+      <c r="U2" t="str">
+        <v>082120018449</v>
+      </c>
+      <c r="V2" t="str">
+        <v>Yayasan</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Global Humanis Indonesia</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Yogie Subagya</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>081210576976</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>globalhumanisindonesia@gmail.com</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Lahan, Bangunan, Alat Makan</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>DKI JAKARTA</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>KOTA ADM. JAKARTA SELATAN</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>KEBAYORAN BARU</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>GANDARIA UTARA</v>
+      </c>
+      <c r="AF2" t="str">
+        <v>Komplek Ruko Radio Dalam Square Nomr 1B</v>
+      </c>
+      <c r="AG2" t="str">
+        <v>12140</v>
+      </c>
+      <c r="AH2" t="str">
+        <v>Yayasan Darma Bandhawa Kulinari</v>
+      </c>
+      <c r="AI2" t="str">
+        <v>1000000003216833</v>
+      </c>
+      <c r="AJ2" t="str">
+        <v>JAWA BARAT</v>
+      </c>
+      <c r="AK2" t="str">
+        <v>KOTA BANDUNG</v>
+      </c>
+      <c r="AL2" t="str">
+        <v>BANDUNG KULON</v>
+      </c>
+      <c r="AM2" t="str">
+        <v>GEMPOL SARI</v>
+      </c>
+      <c r="AN2" t="str">
+        <v>Jl. Gempol Asri Raya No 84, Malausma</v>
+      </c>
+      <c r="AO2" t="str">
+        <v>40215</v>
+      </c>
+      <c r="AP2" t="str">
+        <v>darma.bhandawakulinari@gmail.com</v>
+      </c>
+      <c r="AQ2" t="str">
+        <v>082315167789</v>
+      </c>
+      <c r="AR2" t="str">
+        <v>BANK BNI</v>
+      </c>
+      <c r="AS2" t="str">
+        <v>2917122527</v>
+      </c>
+      <c r="AT2" t="str">
+        <v>Benteng Generasi Mandiri Yayasan</v>
+      </c>
+      <c r="AU2" t="str">
+        <v>BANK BNI</v>
+      </c>
+      <c r="AV2" t="str">
+        <v>5268080020571600</v>
+      </c>
+      <c r="AW2" t="str">
+        <v>205716 OWJZUCPO DARMA BAND (IDR)</v>
+      </c>
+      <c r="AX2" t="str">
+        <v>DEVI NURJAMAN</v>
+      </c>
+      <c r="AY2" t="str">
+        <v>3205121311960006</v>
+      </c>
+      <c r="AZ2" t="str">
+        <v>dnur9414@gmail.com</v>
+      </c>
+      <c r="BA2" t="str">
+        <v>089507760120</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BA2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>